<commit_message>
Updated to latest data
</commit_message>
<xml_diff>
--- a/predictions/model_compare.xlsx
+++ b/predictions/model_compare.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ripa_\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ripa_\Desktop\Programing\IndyCar_Project\predictions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F23E69E-BB1C-4D19-8F4C-0B9BBDE10D37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF2B043F-FAC7-4114-98E9-A1461423C0C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" firstSheet="2" activeTab="2" xr2:uid="{74EB7EE7-EB5C-4423-87E4-FE46F1C4926A}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{74EB7EE7-EB5C-4423-87E4-FE46F1C4926A}"/>
   </bookViews>
   <sheets>
     <sheet name="Pre-Qualy" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="889" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="914" uniqueCount="87">
   <si>
     <t>Model</t>
   </si>
@@ -406,6 +406,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -417,10 +421,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -943,22 +943,22 @@
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="11"/>
-      <c r="D1" s="8" t="s">
+      <c r="C1" s="13"/>
+      <c r="D1" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="8"/>
-      <c r="F1" s="9" t="s">
+      <c r="E1" s="10"/>
+      <c r="F1" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9" t="s">
+      <c r="G1" s="11"/>
+      <c r="H1" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="9"/>
+      <c r="I1" s="11"/>
       <c r="J1" t="s">
         <v>51</v>
       </c>
@@ -1197,22 +1197,22 @@
       <c r="A11" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="11"/>
-      <c r="D11" s="8" t="s">
+      <c r="C11" s="13"/>
+      <c r="D11" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="E11" s="8"/>
-      <c r="F11" s="9" t="s">
+      <c r="E11" s="10"/>
+      <c r="F11" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9" t="s">
+      <c r="G11" s="11"/>
+      <c r="H11" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="I11" s="9"/>
+      <c r="I11" s="11"/>
       <c r="J11" t="s">
         <v>50</v>
       </c>
@@ -1677,22 +1677,22 @@
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="11"/>
-      <c r="D1" s="8" t="s">
+      <c r="C1" s="13"/>
+      <c r="D1" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="8"/>
-      <c r="F1" s="9" t="s">
+      <c r="E1" s="10"/>
+      <c r="F1" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9" t="s">
+      <c r="G1" s="11"/>
+      <c r="H1" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="9"/>
+      <c r="I1" s="11"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="1"/>
@@ -2291,10 +2291,6 @@
       </c>
       <c r="D24">
         <v>0.24890000000000001</v>
-      </c>
-      <c r="F24">
-        <f>C24*25</f>
-        <v>5.2025000000000006</v>
       </c>
     </row>
   </sheetData>
@@ -6434,7 +6430,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O101"/>
+  <dimension ref="A1:O102"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="17.20703125" bestFit="1" customWidth="1"/>
@@ -6494,15 +6490,15 @@
       <c r="A2" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="B2" s="13">
+      <c r="B2" s="9">
         <v>6.23</v>
       </c>
       <c r="C2" s="5">
-        <f>B2-L2</f>
+        <f t="shared" ref="C2:C33" si="0">B2-L2</f>
         <v>1.0300000000000002</v>
       </c>
       <c r="D2" s="5">
-        <f>B2+L2</f>
+        <f t="shared" ref="D2:D33" si="1">B2+L2</f>
         <v>11.43</v>
       </c>
       <c r="E2" s="5">
@@ -6535,15 +6531,15 @@
       <c r="A3" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B3" s="13">
+      <c r="B3" s="9">
         <v>7.33</v>
       </c>
       <c r="C3" s="5">
-        <f>B3-L3</f>
+        <f t="shared" si="0"/>
         <v>2.13</v>
       </c>
       <c r="D3" s="5">
-        <f>B3+L3</f>
+        <f t="shared" si="1"/>
         <v>12.530000000000001</v>
       </c>
       <c r="E3" s="5">
@@ -6576,15 +6572,15 @@
       <c r="A4" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="13">
+      <c r="B4" s="9">
         <v>8.7899999999999991</v>
       </c>
       <c r="C4" s="5">
-        <f>B4-L4</f>
+        <f t="shared" si="0"/>
         <v>3.589999999999999</v>
       </c>
       <c r="D4" s="5">
-        <f>B4+L4</f>
+        <f t="shared" si="1"/>
         <v>13.989999999999998</v>
       </c>
       <c r="E4" s="5">
@@ -6617,15 +6613,15 @@
       <c r="A5" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="13">
+      <c r="B5" s="9">
         <v>8.8000000000000007</v>
       </c>
       <c r="C5" s="5">
-        <f>B5-L5</f>
+        <f t="shared" si="0"/>
         <v>3.6000000000000005</v>
       </c>
       <c r="D5" s="5">
-        <f>B5+L5</f>
+        <f t="shared" si="1"/>
         <v>14</v>
       </c>
       <c r="E5" s="5">
@@ -6658,15 +6654,15 @@
       <c r="A6" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="13">
+      <c r="B6" s="9">
         <v>8.85</v>
       </c>
       <c r="C6" s="5">
-        <f>B6-L6</f>
+        <f t="shared" si="0"/>
         <v>3.6499999999999995</v>
       </c>
       <c r="D6" s="5">
-        <f>B6+L6</f>
+        <f t="shared" si="1"/>
         <v>14.05</v>
       </c>
       <c r="E6" s="5">
@@ -6699,15 +6695,15 @@
       <c r="A7" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="13">
+      <c r="B7" s="9">
         <v>9.3000000000000007</v>
       </c>
       <c r="C7" s="5">
-        <f>B7-L7</f>
+        <f t="shared" si="0"/>
         <v>4.1000000000000005</v>
       </c>
       <c r="D7" s="5">
-        <f>B7+L7</f>
+        <f t="shared" si="1"/>
         <v>14.5</v>
       </c>
       <c r="E7" s="5">
@@ -6740,15 +6736,15 @@
       <c r="A8" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="13">
+      <c r="B8" s="9">
         <v>9.57</v>
       </c>
       <c r="C8" s="5">
-        <f>B8-L8</f>
+        <f t="shared" si="0"/>
         <v>4.37</v>
       </c>
       <c r="D8" s="5">
-        <f>B8+L8</f>
+        <f t="shared" si="1"/>
         <v>14.77</v>
       </c>
       <c r="E8" s="5">
@@ -6781,15 +6777,15 @@
       <c r="A9" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="13">
+      <c r="B9" s="9">
         <v>10.210000000000001</v>
       </c>
       <c r="C9" s="5">
-        <f>B9-L9</f>
+        <f t="shared" si="0"/>
         <v>5.0100000000000007</v>
       </c>
       <c r="D9" s="5">
-        <f>B9+L9</f>
+        <f t="shared" si="1"/>
         <v>15.41</v>
       </c>
       <c r="E9" s="5">
@@ -6822,15 +6818,15 @@
       <c r="A10" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="13">
+      <c r="B10" s="9">
         <v>10.56</v>
       </c>
       <c r="C10" s="5">
-        <f>B10-L10</f>
+        <f t="shared" si="0"/>
         <v>5.36</v>
       </c>
       <c r="D10" s="5">
-        <f>B10+L10</f>
+        <f t="shared" si="1"/>
         <v>15.760000000000002</v>
       </c>
       <c r="E10" s="5">
@@ -6863,15 +6859,15 @@
       <c r="A11" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="B11" s="13">
+      <c r="B11" s="9">
         <v>10.63</v>
       </c>
       <c r="C11" s="5">
-        <f>B11-L11</f>
+        <f t="shared" si="0"/>
         <v>5.4300000000000006</v>
       </c>
       <c r="D11" s="5">
-        <f>B11+L11</f>
+        <f t="shared" si="1"/>
         <v>15.830000000000002</v>
       </c>
       <c r="E11" s="5">
@@ -6904,15 +6900,15 @@
       <c r="A12" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="13">
+      <c r="B12" s="9">
         <v>10.91</v>
       </c>
       <c r="C12" s="5">
-        <f>B12-L12</f>
+        <f t="shared" si="0"/>
         <v>5.71</v>
       </c>
       <c r="D12" s="5">
-        <f>B12+L12</f>
+        <f t="shared" si="1"/>
         <v>16.11</v>
       </c>
       <c r="E12" s="5">
@@ -6945,15 +6941,15 @@
       <c r="A13" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="B13" s="13">
+      <c r="B13" s="9">
         <v>10.95</v>
       </c>
       <c r="C13" s="5">
-        <f>B13-L13</f>
+        <f t="shared" si="0"/>
         <v>5.7499999999999991</v>
       </c>
       <c r="D13" s="5">
-        <f>B13+L13</f>
+        <f t="shared" si="1"/>
         <v>16.149999999999999</v>
       </c>
       <c r="E13" s="5">
@@ -6986,15 +6982,15 @@
       <c r="A14" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B14" s="13">
+      <c r="B14" s="9">
         <v>11.51</v>
       </c>
       <c r="C14" s="5">
-        <f>B14-L14</f>
+        <f t="shared" si="0"/>
         <v>6.31</v>
       </c>
       <c r="D14" s="5">
-        <f>B14+L14</f>
+        <f t="shared" si="1"/>
         <v>16.71</v>
       </c>
       <c r="E14" s="5">
@@ -7027,15 +7023,15 @@
       <c r="A15" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="B15" s="13">
+      <c r="B15" s="9">
         <v>11.97</v>
       </c>
       <c r="C15" s="5">
-        <f>B15-L15</f>
+        <f t="shared" si="0"/>
         <v>6.7700000000000005</v>
       </c>
       <c r="D15" s="5">
-        <f>B15+L15</f>
+        <f t="shared" si="1"/>
         <v>17.170000000000002</v>
       </c>
       <c r="E15" s="5">
@@ -7068,15 +7064,15 @@
       <c r="A16" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B16" s="13">
+      <c r="B16" s="9">
         <v>12.74</v>
       </c>
       <c r="C16" s="5">
-        <f>B16-L16</f>
+        <f t="shared" si="0"/>
         <v>7.54</v>
       </c>
       <c r="D16" s="5">
-        <f>B16+L16</f>
+        <f t="shared" si="1"/>
         <v>17.940000000000001</v>
       </c>
       <c r="E16" s="5">
@@ -7109,15 +7105,15 @@
       <c r="A17" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B17" s="13">
+      <c r="B17" s="9">
         <v>12.75</v>
       </c>
       <c r="C17" s="5">
-        <f>B17-L17</f>
+        <f t="shared" si="0"/>
         <v>7.55</v>
       </c>
       <c r="D17" s="5">
-        <f>B17+L17</f>
+        <f t="shared" si="1"/>
         <v>17.95</v>
       </c>
       <c r="E17" s="5">
@@ -7150,15 +7146,15 @@
       <c r="A18" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="13">
+      <c r="B18" s="9">
         <v>12.94</v>
       </c>
       <c r="C18" s="5">
-        <f>B18-L18</f>
+        <f t="shared" si="0"/>
         <v>7.7399999999999993</v>
       </c>
       <c r="D18" s="5">
-        <f>B18+L18</f>
+        <f t="shared" si="1"/>
         <v>18.14</v>
       </c>
       <c r="E18" s="5">
@@ -7191,15 +7187,15 @@
       <c r="A19" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B19" s="13">
+      <c r="B19" s="9">
         <v>13.76</v>
       </c>
       <c r="C19" s="5">
-        <f>B19-L19</f>
+        <f t="shared" si="0"/>
         <v>8.5599999999999987</v>
       </c>
       <c r="D19" s="5">
-        <f>B19+L19</f>
+        <f t="shared" si="1"/>
         <v>18.96</v>
       </c>
       <c r="E19" s="5">
@@ -7232,15 +7228,15 @@
       <c r="A20" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="B20" s="13">
+      <c r="B20" s="9">
         <v>14.13</v>
       </c>
       <c r="C20" s="5">
-        <f>B20-L20</f>
+        <f t="shared" si="0"/>
         <v>8.93</v>
       </c>
       <c r="D20" s="5">
-        <f>B20+L20</f>
+        <f t="shared" si="1"/>
         <v>19.330000000000002</v>
       </c>
       <c r="E20" s="5">
@@ -7273,15 +7269,15 @@
       <c r="A21" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="B21" s="13">
+      <c r="B21" s="9">
         <v>14.49</v>
       </c>
       <c r="C21" s="5">
-        <f>B21-L21</f>
+        <f t="shared" si="0"/>
         <v>9.2899999999999991</v>
       </c>
       <c r="D21" s="5">
-        <f>B21+L21</f>
+        <f t="shared" si="1"/>
         <v>19.690000000000001</v>
       </c>
       <c r="E21" s="5">
@@ -7314,15 +7310,15 @@
       <c r="A22" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B22" s="13">
+      <c r="B22" s="9">
         <v>14.54</v>
       </c>
       <c r="C22" s="5">
-        <f>B22-L22</f>
+        <f t="shared" si="0"/>
         <v>9.34</v>
       </c>
       <c r="D22" s="5">
-        <f>B22+L22</f>
+        <f t="shared" si="1"/>
         <v>19.739999999999998</v>
       </c>
       <c r="E22" s="5">
@@ -7355,15 +7351,15 @@
       <c r="A23" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="B23" s="13">
+      <c r="B23" s="9">
         <v>15.99</v>
       </c>
       <c r="C23" s="5">
-        <f>B23-L23</f>
+        <f t="shared" si="0"/>
         <v>10.79</v>
       </c>
       <c r="D23" s="5">
-        <f>B23+L23</f>
+        <f t="shared" si="1"/>
         <v>21.19</v>
       </c>
       <c r="E23" s="5">
@@ -7396,15 +7392,15 @@
       <c r="A24" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="B24" s="13">
+      <c r="B24" s="9">
         <v>16.36</v>
       </c>
       <c r="C24" s="5">
-        <f>B24-L24</f>
+        <f t="shared" si="0"/>
         <v>11.16</v>
       </c>
       <c r="D24" s="5">
-        <f>B24+L24</f>
+        <f t="shared" si="1"/>
         <v>21.56</v>
       </c>
       <c r="E24" s="5">
@@ -7437,15 +7433,15 @@
       <c r="A25" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B25" s="13">
+      <c r="B25" s="9">
         <v>17.11</v>
       </c>
       <c r="C25" s="5">
-        <f>B25-L25</f>
+        <f t="shared" si="0"/>
         <v>11.91</v>
       </c>
       <c r="D25" s="5">
-        <f>B25+L25</f>
+        <f t="shared" si="1"/>
         <v>22.31</v>
       </c>
       <c r="E25" s="5">
@@ -7478,15 +7474,15 @@
       <c r="A26" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B26" s="13">
+      <c r="B26" s="9">
         <v>17.440000000000001</v>
       </c>
       <c r="C26" s="5">
-        <f>B26-L26</f>
+        <f t="shared" si="0"/>
         <v>12.240000000000002</v>
       </c>
       <c r="D26" s="5">
-        <f>B26+L26</f>
+        <f t="shared" si="1"/>
         <v>22.64</v>
       </c>
       <c r="E26" s="5">
@@ -7523,11 +7519,11 @@
         <v>8.4700000000000006</v>
       </c>
       <c r="C27" s="5">
-        <f>B27-L27</f>
+        <f t="shared" si="0"/>
         <v>3.1000000000000005</v>
       </c>
       <c r="D27" s="5">
-        <f>B27+L27</f>
+        <f t="shared" si="1"/>
         <v>13.84</v>
       </c>
       <c r="E27" s="5">
@@ -7536,10 +7532,10 @@
       <c r="F27">
         <v>1</v>
       </c>
-      <c r="G27" s="12">
+      <c r="G27" s="8">
         <v>10</v>
       </c>
-      <c r="H27" s="12">
+      <c r="H27" s="8">
         <v>24</v>
       </c>
       <c r="I27" t="s">
@@ -7565,11 +7561,11 @@
         <v>8.59</v>
       </c>
       <c r="C28" s="5">
-        <f>B28-L28</f>
+        <f t="shared" si="0"/>
         <v>3.2199999999999998</v>
       </c>
       <c r="D28" s="5">
-        <f>B28+L28</f>
+        <f t="shared" si="1"/>
         <v>13.96</v>
       </c>
       <c r="E28" s="5">
@@ -7578,10 +7574,10 @@
       <c r="F28">
         <v>2</v>
       </c>
-      <c r="G28" s="12">
+      <c r="G28" s="8">
         <v>1</v>
       </c>
-      <c r="H28" s="12">
+      <c r="H28" s="8">
         <v>8</v>
       </c>
       <c r="I28" t="s">
@@ -7608,11 +7604,11 @@
         <v>9.01</v>
       </c>
       <c r="C29" s="5">
-        <f>B29-L29</f>
+        <f t="shared" si="0"/>
         <v>3.6399999999999997</v>
       </c>
       <c r="D29" s="5">
-        <f>B29+L29</f>
+        <f t="shared" si="1"/>
         <v>14.379999999999999</v>
       </c>
       <c r="E29" s="5">
@@ -7621,10 +7617,10 @@
       <c r="F29">
         <v>3</v>
       </c>
-      <c r="G29" s="12">
+      <c r="G29" s="8">
         <v>2</v>
       </c>
-      <c r="H29" s="12">
+      <c r="H29" s="8">
         <v>4</v>
       </c>
       <c r="I29" t="s">
@@ -7646,15 +7642,15 @@
       <c r="A30" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="B30" s="13">
+      <c r="B30" s="9">
         <v>9.36</v>
       </c>
       <c r="C30" s="5">
-        <f>B30-L30</f>
+        <f t="shared" si="0"/>
         <v>3.9899999999999993</v>
       </c>
       <c r="D30" s="5">
-        <f>B30+L30</f>
+        <f t="shared" si="1"/>
         <v>14.73</v>
       </c>
       <c r="E30" s="5">
@@ -7663,10 +7659,10 @@
       <c r="F30">
         <v>4</v>
       </c>
-      <c r="G30" s="12">
+      <c r="G30" s="8">
         <v>3</v>
       </c>
-      <c r="H30" s="12">
+      <c r="H30" s="8">
         <v>1</v>
       </c>
       <c r="I30" t="s">
@@ -7688,15 +7684,15 @@
       <c r="A31" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B31" s="13">
+      <c r="B31" s="9">
         <v>9.6999999999999993</v>
       </c>
       <c r="C31" s="5">
-        <f>B31-L31</f>
+        <f t="shared" si="0"/>
         <v>4.3299999999999992</v>
       </c>
       <c r="D31" s="5">
-        <f>B31+L31</f>
+        <f t="shared" si="1"/>
         <v>15.07</v>
       </c>
       <c r="E31" s="5">
@@ -7705,10 +7701,10 @@
       <c r="F31">
         <v>5</v>
       </c>
-      <c r="G31" s="12">
+      <c r="G31" s="8">
         <v>4</v>
       </c>
-      <c r="H31" s="12">
+      <c r="H31" s="8">
         <v>9</v>
       </c>
       <c r="I31" t="s">
@@ -7734,11 +7730,11 @@
         <v>9.92</v>
       </c>
       <c r="C32" s="5">
-        <f>B32-L32</f>
+        <f t="shared" si="0"/>
         <v>4.55</v>
       </c>
       <c r="D32" s="5">
-        <f>B32+L32</f>
+        <f t="shared" si="1"/>
         <v>15.29</v>
       </c>
       <c r="E32" s="5">
@@ -7747,10 +7743,10 @@
       <c r="F32">
         <v>6</v>
       </c>
-      <c r="G32" s="12">
+      <c r="G32" s="8">
         <v>5</v>
       </c>
-      <c r="H32" s="12">
+      <c r="H32" s="8">
         <v>7</v>
       </c>
       <c r="I32" t="s">
@@ -7776,11 +7772,11 @@
         <v>10.199999999999999</v>
       </c>
       <c r="C33" s="5">
-        <f>B33-L33</f>
+        <f t="shared" si="0"/>
         <v>4.8299999999999992</v>
       </c>
       <c r="D33" s="5">
-        <f>B33+L33</f>
+        <f t="shared" si="1"/>
         <v>15.57</v>
       </c>
       <c r="E33" s="5">
@@ -7789,10 +7785,10 @@
       <c r="F33">
         <v>7</v>
       </c>
-      <c r="G33" s="12">
+      <c r="G33" s="8">
         <v>18</v>
       </c>
-      <c r="H33" s="12">
+      <c r="H33" s="8">
         <v>18</v>
       </c>
       <c r="I33" t="s">
@@ -7818,11 +7814,11 @@
         <v>10.42</v>
       </c>
       <c r="C34" s="5">
-        <f>B34-L34</f>
+        <f t="shared" ref="C34:C65" si="2">B34-L34</f>
         <v>5.05</v>
       </c>
       <c r="D34" s="5">
-        <f>B34+L34</f>
+        <f t="shared" ref="D34:D65" si="3">B34+L34</f>
         <v>15.79</v>
       </c>
       <c r="E34" s="5">
@@ -7831,10 +7827,10 @@
       <c r="F34">
         <v>8</v>
       </c>
-      <c r="G34" s="12">
+      <c r="G34" s="8">
         <v>6</v>
       </c>
-      <c r="H34" s="12">
+      <c r="H34" s="8">
         <v>2</v>
       </c>
       <c r="I34" t="s">
@@ -7856,15 +7852,15 @@
       <c r="A35" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B35" s="13">
+      <c r="B35" s="9">
         <v>10.57</v>
       </c>
       <c r="C35" s="5">
-        <f>B35-L35</f>
+        <f t="shared" si="2"/>
         <v>5.2</v>
       </c>
       <c r="D35" s="5">
-        <f>B35+L35</f>
+        <f t="shared" si="3"/>
         <v>15.940000000000001</v>
       </c>
       <c r="E35" s="5">
@@ -7873,10 +7869,10 @@
       <c r="F35">
         <v>9</v>
       </c>
-      <c r="G35" s="12">
+      <c r="G35" s="8">
         <v>7</v>
       </c>
-      <c r="H35" s="12">
+      <c r="H35" s="8">
         <v>3</v>
       </c>
       <c r="I35" t="s">
@@ -7902,11 +7898,11 @@
         <v>10.92</v>
       </c>
       <c r="C36" s="5">
-        <f>B36-L36</f>
+        <f t="shared" si="2"/>
         <v>5.55</v>
       </c>
       <c r="D36" s="5">
-        <f>B36+L36</f>
+        <f t="shared" si="3"/>
         <v>16.29</v>
       </c>
       <c r="E36" s="5">
@@ -7915,10 +7911,10 @@
       <c r="F36">
         <v>10</v>
       </c>
-      <c r="G36" s="12">
+      <c r="G36" s="8">
         <v>8</v>
       </c>
-      <c r="H36" s="12">
+      <c r="H36" s="8">
         <v>6</v>
       </c>
       <c r="I36" t="s">
@@ -7944,11 +7940,11 @@
         <v>11.64</v>
       </c>
       <c r="C37" s="5">
-        <f>B37-L37</f>
+        <f t="shared" si="2"/>
         <v>6.2700000000000005</v>
       </c>
       <c r="D37" s="5">
-        <f>B37+L37</f>
+        <f t="shared" si="3"/>
         <v>17.010000000000002</v>
       </c>
       <c r="E37" s="5">
@@ -7957,10 +7953,10 @@
       <c r="F37">
         <v>11</v>
       </c>
-      <c r="G37" s="12">
+      <c r="G37" s="8">
         <v>19</v>
       </c>
-      <c r="H37" s="12">
+      <c r="H37" s="8">
         <v>17</v>
       </c>
       <c r="I37" t="s">
@@ -7986,11 +7982,11 @@
         <v>11.74</v>
       </c>
       <c r="C38" s="5">
-        <f>B38-L38</f>
+        <f t="shared" si="2"/>
         <v>6.37</v>
       </c>
       <c r="D38" s="5">
-        <f>B38+L38</f>
+        <f t="shared" si="3"/>
         <v>17.11</v>
       </c>
       <c r="E38" s="5">
@@ -7999,10 +7995,10 @@
       <c r="F38">
         <v>12</v>
       </c>
-      <c r="G38" s="12">
+      <c r="G38" s="8">
         <v>12</v>
       </c>
-      <c r="H38" s="12">
+      <c r="H38" s="8">
         <v>16</v>
       </c>
       <c r="I38" t="s">
@@ -8028,11 +8024,11 @@
         <v>11.91</v>
       </c>
       <c r="C39" s="5">
-        <f>B39-L39</f>
+        <f t="shared" si="2"/>
         <v>6.54</v>
       </c>
       <c r="D39" s="5">
-        <f>B39+L39</f>
+        <f t="shared" si="3"/>
         <v>17.28</v>
       </c>
       <c r="E39" s="5">
@@ -8041,10 +8037,10 @@
       <c r="F39">
         <v>13</v>
       </c>
-      <c r="G39" s="12">
+      <c r="G39" s="8">
         <v>13</v>
       </c>
-      <c r="H39" s="12">
+      <c r="H39" s="8">
         <v>22</v>
       </c>
       <c r="I39" t="s">
@@ -8070,11 +8066,11 @@
         <v>12.23</v>
       </c>
       <c r="C40" s="5">
-        <f>B40-L40</f>
+        <f t="shared" si="2"/>
         <v>6.86</v>
       </c>
       <c r="D40" s="5">
-        <f>B40+L40</f>
+        <f t="shared" si="3"/>
         <v>17.600000000000001</v>
       </c>
       <c r="E40" s="5">
@@ -8083,10 +8079,10 @@
       <c r="F40">
         <v>14</v>
       </c>
-      <c r="G40" s="12">
+      <c r="G40" s="8">
         <v>20</v>
       </c>
-      <c r="H40" s="12">
+      <c r="H40" s="8">
         <v>13</v>
       </c>
       <c r="I40" t="s">
@@ -8112,11 +8108,11 @@
         <v>12.83</v>
       </c>
       <c r="C41" s="5">
-        <f>B41-L41</f>
+        <f t="shared" si="2"/>
         <v>7.46</v>
       </c>
       <c r="D41" s="5">
-        <f>B41+L41</f>
+        <f t="shared" si="3"/>
         <v>18.2</v>
       </c>
       <c r="E41" s="5">
@@ -8125,10 +8121,10 @@
       <c r="F41">
         <v>15</v>
       </c>
-      <c r="G41" s="12">
+      <c r="G41" s="8">
         <v>9</v>
       </c>
-      <c r="H41" s="12">
+      <c r="H41" s="8">
         <v>5</v>
       </c>
       <c r="I41" t="s">
@@ -8154,11 +8150,11 @@
         <v>13.29</v>
       </c>
       <c r="C42" s="5">
-        <f>B42-L42</f>
+        <f t="shared" si="2"/>
         <v>7.919999999999999</v>
       </c>
       <c r="D42" s="5">
-        <f>B42+L42</f>
+        <f t="shared" si="3"/>
         <v>18.66</v>
       </c>
       <c r="E42" s="5">
@@ -8167,10 +8163,10 @@
       <c r="F42">
         <v>16</v>
       </c>
-      <c r="G42" s="12">
+      <c r="G42" s="8">
         <v>21</v>
       </c>
-      <c r="H42" s="12">
+      <c r="H42" s="8">
         <v>20</v>
       </c>
       <c r="I42" t="s">
@@ -8196,11 +8192,11 @@
         <v>13.91</v>
       </c>
       <c r="C43" s="5">
-        <f>B43-L43</f>
+        <f t="shared" si="2"/>
         <v>8.5399999999999991</v>
       </c>
       <c r="D43" s="5">
-        <f>B43+L43</f>
+        <f t="shared" si="3"/>
         <v>19.28</v>
       </c>
       <c r="E43" s="5">
@@ -8209,10 +8205,10 @@
       <c r="F43">
         <v>17</v>
       </c>
-      <c r="G43" s="12">
+      <c r="G43" s="8">
         <v>14</v>
       </c>
-      <c r="H43" s="12">
+      <c r="H43" s="8">
         <v>12</v>
       </c>
       <c r="I43" t="s">
@@ -8238,11 +8234,11 @@
         <v>14.26</v>
       </c>
       <c r="C44" s="5">
-        <f>B44-L44</f>
+        <f t="shared" si="2"/>
         <v>8.89</v>
       </c>
       <c r="D44" s="5">
-        <f>B44+L44</f>
+        <f t="shared" si="3"/>
         <v>19.63</v>
       </c>
       <c r="E44" s="5">
@@ -8251,10 +8247,10 @@
       <c r="F44">
         <v>18</v>
       </c>
-      <c r="G44" s="12">
+      <c r="G44" s="8">
         <v>15</v>
       </c>
-      <c r="H44" s="12">
+      <c r="H44" s="8">
         <v>11</v>
       </c>
       <c r="I44" t="s">
@@ -8280,11 +8276,11 @@
         <v>14.5</v>
       </c>
       <c r="C45" s="5">
-        <f>B45-L45</f>
+        <f t="shared" si="2"/>
         <v>9.129999999999999</v>
       </c>
       <c r="D45" s="5">
-        <f>B45+L45</f>
+        <f t="shared" si="3"/>
         <v>19.87</v>
       </c>
       <c r="E45" s="5">
@@ -8293,10 +8289,10 @@
       <c r="F45">
         <v>19</v>
       </c>
-      <c r="G45" s="12">
+      <c r="G45" s="8">
         <v>22</v>
       </c>
-      <c r="H45" s="12">
+      <c r="H45" s="8">
         <v>15</v>
       </c>
       <c r="I45" t="s">
@@ -8322,11 +8318,11 @@
         <v>14.76</v>
       </c>
       <c r="C46" s="5">
-        <f>B46-L46</f>
+        <f t="shared" si="2"/>
         <v>9.39</v>
       </c>
       <c r="D46" s="5">
-        <f>B46+L46</f>
+        <f t="shared" si="3"/>
         <v>20.13</v>
       </c>
       <c r="E46" s="5">
@@ -8335,10 +8331,10 @@
       <c r="F46">
         <v>20</v>
       </c>
-      <c r="G46" s="12">
+      <c r="G46" s="8">
         <v>13</v>
       </c>
-      <c r="H46" s="12">
+      <c r="H46" s="8">
         <v>19</v>
       </c>
       <c r="I46" t="s">
@@ -8364,11 +8360,11 @@
         <v>14.91</v>
       </c>
       <c r="C47" s="5">
-        <f>B47-L47</f>
+        <f t="shared" si="2"/>
         <v>9.5399999999999991</v>
       </c>
       <c r="D47" s="5">
-        <f>B47+L47</f>
+        <f t="shared" si="3"/>
         <v>20.28</v>
       </c>
       <c r="E47" s="5">
@@ -8377,10 +8373,10 @@
       <c r="F47">
         <v>21</v>
       </c>
-      <c r="G47" s="12">
+      <c r="G47" s="8">
         <v>16</v>
       </c>
-      <c r="H47" s="12">
+      <c r="H47" s="8">
         <v>25</v>
       </c>
       <c r="I47" t="s">
@@ -8406,11 +8402,11 @@
         <v>14.93</v>
       </c>
       <c r="C48" s="5">
-        <f>B48-L48</f>
+        <f t="shared" si="2"/>
         <v>9.5599999999999987</v>
       </c>
       <c r="D48" s="5">
-        <f>B48+L48</f>
+        <f t="shared" si="3"/>
         <v>20.3</v>
       </c>
       <c r="E48" s="5">
@@ -8419,10 +8415,10 @@
       <c r="F48">
         <v>22</v>
       </c>
-      <c r="G48" s="12">
+      <c r="G48" s="8">
         <v>24</v>
       </c>
-      <c r="H48" s="12">
+      <c r="H48" s="8">
         <v>21</v>
       </c>
       <c r="I48" t="s">
@@ -8448,11 +8444,11 @@
         <v>14.99</v>
       </c>
       <c r="C49" s="5">
-        <f>B49-L49</f>
+        <f t="shared" si="2"/>
         <v>9.620000000000001</v>
       </c>
       <c r="D49" s="5">
-        <f>B49+L49</f>
+        <f t="shared" si="3"/>
         <v>20.36</v>
       </c>
       <c r="E49" s="5">
@@ -8461,10 +8457,10 @@
       <c r="F49">
         <v>23</v>
       </c>
-      <c r="G49" s="12">
+      <c r="G49" s="8">
         <v>17</v>
       </c>
-      <c r="H49" s="12">
+      <c r="H49" s="8">
         <v>23</v>
       </c>
       <c r="I49" t="s">
@@ -8490,11 +8486,11 @@
         <v>15.02</v>
       </c>
       <c r="C50" s="5">
-        <f>B50-L50</f>
+        <f t="shared" si="2"/>
         <v>9.6499999999999986</v>
       </c>
       <c r="D50" s="5">
-        <f>B50+L50</f>
+        <f t="shared" si="3"/>
         <v>20.39</v>
       </c>
       <c r="E50" s="5">
@@ -8503,10 +8499,10 @@
       <c r="F50">
         <v>24</v>
       </c>
-      <c r="G50" s="12">
+      <c r="G50" s="8">
         <v>25</v>
       </c>
-      <c r="H50" s="12">
+      <c r="H50" s="8">
         <v>10</v>
       </c>
       <c r="I50" t="s">
@@ -8532,11 +8528,11 @@
         <v>15.76</v>
       </c>
       <c r="C51" s="5">
-        <f>B51-L51</f>
+        <f t="shared" si="2"/>
         <v>10.39</v>
       </c>
       <c r="D51" s="5">
-        <f>B51+L51</f>
+        <f t="shared" si="3"/>
         <v>21.13</v>
       </c>
       <c r="E51" s="5">
@@ -8545,10 +8541,10 @@
       <c r="F51">
         <v>25</v>
       </c>
-      <c r="G51" s="12">
+      <c r="G51" s="8">
         <v>11</v>
       </c>
-      <c r="H51" s="12">
+      <c r="H51" s="8">
         <v>14</v>
       </c>
       <c r="I51" t="s">
@@ -8574,11 +8570,11 @@
         <v>7.18</v>
       </c>
       <c r="C52" s="5">
-        <f>B52-L52</f>
+        <f t="shared" si="2"/>
         <v>1.8199999999999994</v>
       </c>
       <c r="D52" s="5">
-        <f>B52+L52</f>
+        <f t="shared" si="3"/>
         <v>12.54</v>
       </c>
       <c r="E52" s="5">
@@ -8587,10 +8583,10 @@
       <c r="F52">
         <v>1</v>
       </c>
-      <c r="G52" s="12">
+      <c r="G52" s="8">
         <v>1</v>
       </c>
-      <c r="H52" s="12">
+      <c r="H52" s="8">
         <v>5</v>
       </c>
       <c r="I52" t="s">
@@ -8616,11 +8612,11 @@
         <v>8.57</v>
       </c>
       <c r="C53" s="5">
-        <f>B53-L53</f>
+        <f t="shared" si="2"/>
         <v>3.21</v>
       </c>
       <c r="D53" s="5">
-        <f>B53+L53</f>
+        <f t="shared" si="3"/>
         <v>13.93</v>
       </c>
       <c r="E53" s="5">
@@ -8629,10 +8625,10 @@
       <c r="F53">
         <v>2</v>
       </c>
-      <c r="G53" s="12">
+      <c r="G53" s="8">
         <v>11</v>
       </c>
-      <c r="H53" s="12">
+      <c r="H53" s="8">
         <v>4</v>
       </c>
       <c r="I53" t="s">
@@ -8656,11 +8652,11 @@
         <v>8.65</v>
       </c>
       <c r="C54" s="5">
-        <f>B54-L54</f>
+        <f t="shared" si="2"/>
         <v>3.29</v>
       </c>
       <c r="D54" s="5">
-        <f>B54+L54</f>
+        <f t="shared" si="3"/>
         <v>14.010000000000002</v>
       </c>
       <c r="E54" s="5">
@@ -8669,10 +8665,10 @@
       <c r="F54">
         <v>3</v>
       </c>
-      <c r="G54" s="12">
+      <c r="G54" s="8">
         <v>2</v>
       </c>
-      <c r="H54" s="12">
+      <c r="H54" s="8">
         <v>2</v>
       </c>
       <c r="I54" t="s">
@@ -8696,11 +8692,11 @@
         <v>9.17</v>
       </c>
       <c r="C55" s="5">
-        <f>B55-L55</f>
+        <f t="shared" si="2"/>
         <v>3.8099999999999996</v>
       </c>
       <c r="D55" s="5">
-        <f>B55+L55</f>
+        <f t="shared" si="3"/>
         <v>14.530000000000001</v>
       </c>
       <c r="E55" s="5">
@@ -8709,10 +8705,10 @@
       <c r="F55">
         <v>4</v>
       </c>
-      <c r="G55" s="12">
+      <c r="G55" s="8">
         <v>3</v>
       </c>
-      <c r="H55" s="12"/>
+      <c r="H55" s="8"/>
       <c r="I55" t="s">
         <v>81</v>
       </c>
@@ -8734,11 +8730,11 @@
         <v>9.18</v>
       </c>
       <c r="C56" s="5">
-        <f>B56-L56</f>
+        <f t="shared" si="2"/>
         <v>3.8199999999999994</v>
       </c>
       <c r="D56" s="5">
-        <f>B56+L56</f>
+        <f t="shared" si="3"/>
         <v>14.54</v>
       </c>
       <c r="E56" s="5">
@@ -8747,10 +8743,10 @@
       <c r="F56">
         <v>5</v>
       </c>
-      <c r="G56" s="12">
+      <c r="G56" s="8">
         <v>4</v>
       </c>
-      <c r="H56" s="12">
+      <c r="H56" s="8">
         <v>3</v>
       </c>
       <c r="I56" t="s">
@@ -8774,11 +8770,11 @@
         <v>9.31</v>
       </c>
       <c r="C57" s="5">
-        <f>B57-L57</f>
+        <f t="shared" si="2"/>
         <v>3.95</v>
       </c>
       <c r="D57" s="5">
-        <f>B57+L57</f>
+        <f t="shared" si="3"/>
         <v>14.670000000000002</v>
       </c>
       <c r="E57" s="5">
@@ -8787,10 +8783,10 @@
       <c r="F57">
         <v>6</v>
       </c>
-      <c r="G57" s="12">
+      <c r="G57" s="8">
         <v>5</v>
       </c>
-      <c r="H57" s="12">
+      <c r="H57" s="8">
         <v>1</v>
       </c>
       <c r="I57" t="s">
@@ -8814,11 +8810,11 @@
         <v>9.5500000000000007</v>
       </c>
       <c r="C58" s="5">
-        <f>B58-L58</f>
+        <f t="shared" si="2"/>
         <v>4.1900000000000004</v>
       </c>
       <c r="D58" s="5">
-        <f>B58+L58</f>
+        <f t="shared" si="3"/>
         <v>14.91</v>
       </c>
       <c r="E58" s="5">
@@ -8827,10 +8823,10 @@
       <c r="F58">
         <v>7</v>
       </c>
-      <c r="G58" s="12">
+      <c r="G58" s="8">
         <v>6</v>
       </c>
-      <c r="H58" s="12">
+      <c r="H58" s="8">
         <v>15</v>
       </c>
       <c r="I58" t="s">
@@ -8854,11 +8850,11 @@
         <v>9.65</v>
       </c>
       <c r="C59" s="5">
-        <f>B59-L59</f>
+        <f t="shared" si="2"/>
         <v>4.29</v>
       </c>
       <c r="D59" s="5">
-        <f>B59+L59</f>
+        <f t="shared" si="3"/>
         <v>15.010000000000002</v>
       </c>
       <c r="E59" s="5">
@@ -8867,10 +8863,10 @@
       <c r="F59">
         <v>8</v>
       </c>
-      <c r="G59" s="12">
+      <c r="G59" s="8">
         <v>7</v>
       </c>
-      <c r="H59" s="12">
+      <c r="H59" s="8">
         <v>8</v>
       </c>
       <c r="I59" t="s">
@@ -8894,11 +8890,11 @@
         <v>10.06</v>
       </c>
       <c r="C60" s="5">
-        <f>B60-L60</f>
+        <f t="shared" si="2"/>
         <v>4.7</v>
       </c>
       <c r="D60" s="5">
-        <f>B60+L60</f>
+        <f t="shared" si="3"/>
         <v>15.420000000000002</v>
       </c>
       <c r="E60" s="5">
@@ -8907,10 +8903,10 @@
       <c r="F60">
         <v>9</v>
       </c>
-      <c r="G60" s="12">
+      <c r="G60" s="8">
         <v>12</v>
       </c>
-      <c r="H60" s="12">
+      <c r="H60" s="8">
         <v>10</v>
       </c>
       <c r="I60" t="s">
@@ -8934,11 +8930,11 @@
         <v>10.72</v>
       </c>
       <c r="C61" s="5">
-        <f>B61-L61</f>
+        <f t="shared" si="2"/>
         <v>5.36</v>
       </c>
       <c r="D61" s="5">
-        <f>B61+L61</f>
+        <f t="shared" si="3"/>
         <v>16.080000000000002</v>
       </c>
       <c r="E61" s="5">
@@ -8947,10 +8943,10 @@
       <c r="F61">
         <v>10</v>
       </c>
-      <c r="G61" s="12">
+      <c r="G61" s="8">
         <v>8</v>
       </c>
-      <c r="H61" s="12">
+      <c r="H61" s="8">
         <v>6</v>
       </c>
       <c r="I61" t="s">
@@ -8974,11 +8970,11 @@
         <v>10.73</v>
       </c>
       <c r="C62" s="5">
-        <f>B62-L62</f>
+        <f t="shared" si="2"/>
         <v>5.37</v>
       </c>
       <c r="D62" s="5">
-        <f>B62+L62</f>
+        <f t="shared" si="3"/>
         <v>16.09</v>
       </c>
       <c r="E62" s="5">
@@ -8987,10 +8983,10 @@
       <c r="F62">
         <v>11</v>
       </c>
-      <c r="G62" s="12">
+      <c r="G62" s="8">
         <v>9</v>
       </c>
-      <c r="H62" s="12">
+      <c r="H62" s="8">
         <v>7</v>
       </c>
       <c r="I62" t="s">
@@ -9014,11 +9010,11 @@
         <v>11.14</v>
       </c>
       <c r="C63" s="5">
-        <f>B63-L63</f>
+        <f t="shared" si="2"/>
         <v>5.78</v>
       </c>
       <c r="D63" s="5">
-        <f>B63+L63</f>
+        <f t="shared" si="3"/>
         <v>16.5</v>
       </c>
       <c r="E63" s="5">
@@ -9027,10 +9023,10 @@
       <c r="F63">
         <v>12</v>
       </c>
-      <c r="G63" s="12">
+      <c r="G63" s="8">
         <v>13</v>
       </c>
-      <c r="H63" s="12">
+      <c r="H63" s="8">
         <v>9</v>
       </c>
       <c r="I63" t="s">
@@ -9054,11 +9050,11 @@
         <v>11.24</v>
       </c>
       <c r="C64" s="5">
-        <f>B64-L64</f>
+        <f t="shared" si="2"/>
         <v>5.88</v>
       </c>
       <c r="D64" s="5">
-        <f>B64+L64</f>
+        <f t="shared" si="3"/>
         <v>16.600000000000001</v>
       </c>
       <c r="E64" s="5">
@@ -9067,10 +9063,10 @@
       <c r="F64">
         <v>13</v>
       </c>
-      <c r="G64" s="12">
+      <c r="G64" s="8">
         <v>14</v>
       </c>
-      <c r="H64" s="12">
+      <c r="H64" s="8">
         <v>11</v>
       </c>
       <c r="I64" t="s">
@@ -9086,7 +9082,7 @@
         <v>5.36</v>
       </c>
     </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+    <row r="65" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" t="s">
         <v>42</v>
       </c>
@@ -9094,11 +9090,11 @@
         <v>12.25</v>
       </c>
       <c r="C65" s="5">
-        <f>B65-L65</f>
+        <f t="shared" si="2"/>
         <v>6.89</v>
       </c>
       <c r="D65" s="5">
-        <f>B65+L65</f>
+        <f t="shared" si="3"/>
         <v>17.61</v>
       </c>
       <c r="E65" s="5">
@@ -9107,10 +9103,10 @@
       <c r="F65">
         <v>14</v>
       </c>
-      <c r="G65" s="12">
+      <c r="G65" s="8">
         <v>18</v>
       </c>
-      <c r="H65" s="12">
+      <c r="H65" s="8">
         <v>25</v>
       </c>
       <c r="I65" t="s">
@@ -9126,7 +9122,7 @@
         <v>5.36</v>
       </c>
     </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+    <row r="66" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" t="s">
         <v>48</v>
       </c>
@@ -9134,11 +9130,11 @@
         <v>12.39</v>
       </c>
       <c r="C66" s="5">
-        <f>B66-L66</f>
+        <f t="shared" ref="C66:C97" si="4">B66-L66</f>
         <v>7.03</v>
       </c>
       <c r="D66" s="5">
-        <f>B66+L66</f>
+        <f t="shared" ref="D66:D101" si="5">B66+L66</f>
         <v>17.75</v>
       </c>
       <c r="E66" s="5">
@@ -9147,10 +9143,10 @@
       <c r="F66">
         <v>15</v>
       </c>
-      <c r="G66" s="12">
+      <c r="G66" s="8">
         <v>10</v>
       </c>
-      <c r="H66" s="12">
+      <c r="H66" s="8">
         <v>19</v>
       </c>
       <c r="I66" t="s">
@@ -9166,7 +9162,7 @@
         <v>5.36</v>
       </c>
     </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+    <row r="67" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A67" t="s">
         <v>30</v>
       </c>
@@ -9174,11 +9170,11 @@
         <v>13.02</v>
       </c>
       <c r="C67" s="5">
-        <f>B67-L67</f>
+        <f t="shared" si="4"/>
         <v>7.6599999999999993</v>
       </c>
       <c r="D67" s="5">
-        <f>B67+L67</f>
+        <f t="shared" si="5"/>
         <v>18.38</v>
       </c>
       <c r="E67" s="5">
@@ -9187,10 +9183,10 @@
       <c r="F67">
         <v>16</v>
       </c>
-      <c r="G67" s="12">
+      <c r="G67" s="8">
         <v>15</v>
       </c>
-      <c r="H67" s="12">
+      <c r="H67" s="8">
         <v>13</v>
       </c>
       <c r="I67" t="s">
@@ -9206,7 +9202,7 @@
         <v>5.36</v>
       </c>
     </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A68" t="s">
         <v>31</v>
       </c>
@@ -9214,11 +9210,11 @@
         <v>13.16</v>
       </c>
       <c r="C68" s="5">
-        <f>B68-L68</f>
+        <f t="shared" si="4"/>
         <v>7.8</v>
       </c>
       <c r="D68" s="5">
-        <f>B68+L68</f>
+        <f t="shared" si="5"/>
         <v>18.52</v>
       </c>
       <c r="E68" s="5">
@@ -9227,10 +9223,10 @@
       <c r="F68">
         <v>17</v>
       </c>
-      <c r="G68" s="12">
+      <c r="G68" s="8">
         <v>16</v>
       </c>
-      <c r="H68" s="12">
+      <c r="H68" s="8">
         <v>23</v>
       </c>
       <c r="I68" t="s">
@@ -9246,7 +9242,7 @@
         <v>5.36</v>
       </c>
     </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+    <row r="69" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A69" t="s">
         <v>41</v>
       </c>
@@ -9254,11 +9250,11 @@
         <v>13.66</v>
       </c>
       <c r="C69" s="5">
-        <f>B69-L69</f>
+        <f t="shared" si="4"/>
         <v>8.3000000000000007</v>
       </c>
       <c r="D69" s="5">
-        <f>B69+L69</f>
+        <f t="shared" si="5"/>
         <v>19.02</v>
       </c>
       <c r="E69" s="5">
@@ -9267,10 +9263,10 @@
       <c r="F69">
         <v>18</v>
       </c>
-      <c r="G69" s="12">
+      <c r="G69" s="8">
         <v>17</v>
       </c>
-      <c r="H69" s="12">
+      <c r="H69" s="8">
         <v>18</v>
       </c>
       <c r="I69" t="s">
@@ -9286,7 +9282,7 @@
         <v>5.36</v>
       </c>
     </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+    <row r="70" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A70" t="s">
         <v>29</v>
       </c>
@@ -9294,11 +9290,11 @@
         <v>14.2</v>
       </c>
       <c r="C70" s="5">
-        <f>B70-L70</f>
+        <f t="shared" si="4"/>
         <v>8.84</v>
       </c>
       <c r="D70" s="5">
-        <f>B70+L70</f>
+        <f t="shared" si="5"/>
         <v>19.559999999999999</v>
       </c>
       <c r="E70" s="5">
@@ -9307,10 +9303,10 @@
       <c r="F70">
         <v>19</v>
       </c>
-      <c r="G70" s="12">
+      <c r="G70" s="8">
         <v>19</v>
       </c>
-      <c r="H70" s="12">
+      <c r="H70" s="8">
         <v>17</v>
       </c>
       <c r="I70" t="s">
@@ -9326,7 +9322,7 @@
         <v>5.36</v>
       </c>
     </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+    <row r="71" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A71" t="s">
         <v>49</v>
       </c>
@@ -9334,11 +9330,11 @@
         <v>14.4</v>
       </c>
       <c r="C71" s="5">
-        <f>B71-L71</f>
+        <f t="shared" si="4"/>
         <v>9.0399999999999991</v>
       </c>
       <c r="D71" s="5">
-        <f>B71+L71</f>
+        <f t="shared" si="5"/>
         <v>19.760000000000002</v>
       </c>
       <c r="E71" s="5">
@@ -9347,10 +9343,10 @@
       <c r="F71">
         <v>20</v>
       </c>
-      <c r="G71" s="12">
+      <c r="G71" s="8">
         <v>20</v>
       </c>
-      <c r="H71" s="12">
+      <c r="H71" s="8">
         <v>14</v>
       </c>
       <c r="I71" t="s">
@@ -9366,7 +9362,7 @@
         <v>5.36</v>
       </c>
     </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+    <row r="72" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A72" t="s">
         <v>47</v>
       </c>
@@ -9374,11 +9370,11 @@
         <v>15.16</v>
       </c>
       <c r="C72" s="5">
-        <f>B72-L72</f>
+        <f t="shared" si="4"/>
         <v>9.8000000000000007</v>
       </c>
       <c r="D72" s="5">
-        <f>B72+L72</f>
+        <f t="shared" si="5"/>
         <v>20.52</v>
       </c>
       <c r="E72" s="5">
@@ -9387,10 +9383,10 @@
       <c r="F72">
         <v>21</v>
       </c>
-      <c r="G72" s="12">
+      <c r="G72" s="8">
         <v>21</v>
       </c>
-      <c r="H72" s="12">
+      <c r="H72" s="8">
         <v>24</v>
       </c>
       <c r="I72" t="s">
@@ -9406,7 +9402,7 @@
         <v>5.36</v>
       </c>
     </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+    <row r="73" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A73" t="s">
         <v>32</v>
       </c>
@@ -9414,11 +9410,11 @@
         <v>15.34</v>
       </c>
       <c r="C73" s="5">
-        <f>B73-L73</f>
+        <f t="shared" si="4"/>
         <v>9.98</v>
       </c>
       <c r="D73" s="5">
-        <f>B73+L73</f>
+        <f t="shared" si="5"/>
         <v>20.7</v>
       </c>
       <c r="E73" s="5">
@@ -9427,10 +9423,10 @@
       <c r="F73">
         <v>22</v>
       </c>
-      <c r="G73" s="12">
+      <c r="G73" s="8">
         <v>22</v>
       </c>
-      <c r="H73" s="12">
+      <c r="H73" s="8">
         <v>16</v>
       </c>
       <c r="I73" t="s">
@@ -9446,7 +9442,7 @@
         <v>5.36</v>
       </c>
     </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+    <row r="74" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A74" t="s">
         <v>26</v>
       </c>
@@ -9454,11 +9450,11 @@
         <v>15.57</v>
       </c>
       <c r="C74" s="5">
-        <f>B74-L74</f>
+        <f t="shared" si="4"/>
         <v>10.210000000000001</v>
       </c>
       <c r="D74" s="5">
-        <f>B74+L74</f>
+        <f t="shared" si="5"/>
         <v>20.93</v>
       </c>
       <c r="E74" s="5">
@@ -9467,10 +9463,10 @@
       <c r="F74">
         <v>23</v>
       </c>
-      <c r="G74" s="12">
+      <c r="G74" s="8">
         <v>23</v>
       </c>
-      <c r="H74" s="12">
+      <c r="H74" s="8">
         <v>12</v>
       </c>
       <c r="I74" t="s">
@@ -9486,7 +9482,7 @@
         <v>5.36</v>
       </c>
     </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+    <row r="75" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A75" t="s">
         <v>46</v>
       </c>
@@ -9494,11 +9490,11 @@
         <v>16.53</v>
       </c>
       <c r="C75" s="5">
-        <f>B75-L75</f>
+        <f t="shared" si="4"/>
         <v>11.170000000000002</v>
       </c>
       <c r="D75" s="5">
-        <f>B75+L75</f>
+        <f t="shared" si="5"/>
         <v>21.89</v>
       </c>
       <c r="E75" s="5">
@@ -9507,10 +9503,10 @@
       <c r="F75">
         <v>24</v>
       </c>
-      <c r="G75" s="12">
+      <c r="G75" s="8">
         <v>24</v>
       </c>
-      <c r="H75" s="12">
+      <c r="H75" s="8">
         <v>22</v>
       </c>
       <c r="I75" t="s">
@@ -9526,7 +9522,7 @@
         <v>5.36</v>
       </c>
     </row>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+    <row r="76" spans="1:15" x14ac:dyDescent="0.55000000000000004">
       <c r="A76" t="s">
         <v>43</v>
       </c>
@@ -9534,11 +9530,11 @@
         <v>17.59</v>
       </c>
       <c r="C76" s="5">
-        <f>B76-L76</f>
+        <f t="shared" si="4"/>
         <v>12.23</v>
       </c>
       <c r="D76" s="5">
-        <f>B76+L76</f>
+        <f t="shared" si="5"/>
         <v>22.95</v>
       </c>
       <c r="E76" s="5">
@@ -9547,10 +9543,10 @@
       <c r="F76">
         <v>25</v>
       </c>
-      <c r="G76" s="12">
+      <c r="G76" s="8">
         <v>25</v>
       </c>
-      <c r="H76" s="12">
+      <c r="H76" s="8">
         <v>21</v>
       </c>
       <c r="I76" t="s">
@@ -9566,22 +9562,33 @@
         <v>5.36</v>
       </c>
     </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="B77" s="5"/>
+    <row r="77" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A77" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B77" s="6">
+        <v>5.63</v>
+      </c>
       <c r="C77" s="5">
-        <f>B77-L77</f>
-        <v>-5.2</v>
+        <f t="shared" si="4"/>
+        <v>0.42999999999999972</v>
       </c>
       <c r="D77" s="5">
-        <f>B77+L77</f>
-        <v>5.2</v>
-      </c>
-      <c r="E77" s="5"/>
+        <f t="shared" si="5"/>
+        <v>10.83</v>
+      </c>
+      <c r="E77" s="5">
+        <v>0.43</v>
+      </c>
       <c r="F77">
         <v>1</v>
       </c>
-      <c r="G77" s="12"/>
-      <c r="H77" s="12"/>
+      <c r="G77" s="8">
+        <v>1</v>
+      </c>
+      <c r="H77" s="8">
+        <v>1</v>
+      </c>
       <c r="I77" t="s">
         <v>75</v>
       </c>
@@ -9595,22 +9602,33 @@
         <v>5.2</v>
       </c>
     </row>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="B78" s="5"/>
+    <row r="78" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A78" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B78" s="6">
+        <v>7.95</v>
+      </c>
       <c r="C78" s="5">
-        <f>B78-L78</f>
-        <v>-5.2</v>
+        <f t="shared" si="4"/>
+        <v>2.75</v>
       </c>
       <c r="D78" s="5">
-        <f>B78+L78</f>
-        <v>5.2</v>
-      </c>
-      <c r="E78" s="5"/>
+        <f t="shared" si="5"/>
+        <v>13.15</v>
+      </c>
+      <c r="E78" s="5">
+        <v>7.95</v>
+      </c>
       <c r="F78">
         <v>2</v>
       </c>
-      <c r="G78" s="12"/>
-      <c r="H78" s="12"/>
+      <c r="G78" s="8">
+        <v>8</v>
+      </c>
+      <c r="H78" s="8">
+        <v>6</v>
+      </c>
       <c r="I78" t="s">
         <v>75</v>
       </c>
@@ -9623,23 +9641,36 @@
       <c r="L78" s="5">
         <v>5.2</v>
       </c>
-    </row>
-    <row r="79" spans="1:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="B79" s="5"/>
+      <c r="N78" s="6"/>
+      <c r="O78" s="5"/>
+    </row>
+    <row r="79" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A79" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B79" s="6">
+        <v>8.39</v>
+      </c>
       <c r="C79" s="5">
-        <f>B79-L79</f>
-        <v>-5.2</v>
+        <f t="shared" si="4"/>
+        <v>3.1900000000000004</v>
       </c>
       <c r="D79" s="5">
-        <f>B79+L79</f>
-        <v>5.2</v>
-      </c>
-      <c r="E79" s="5"/>
+        <f t="shared" si="5"/>
+        <v>13.59</v>
+      </c>
+      <c r="E79" s="5">
+        <v>3.19</v>
+      </c>
       <c r="F79">
         <v>3</v>
       </c>
-      <c r="G79" s="12"/>
-      <c r="H79" s="12"/>
+      <c r="G79" s="8">
+        <v>2</v>
+      </c>
+      <c r="H79" s="8">
+        <v>4</v>
+      </c>
       <c r="I79" t="s">
         <v>75</v>
       </c>
@@ -9652,23 +9683,36 @@
       <c r="L79" s="5">
         <v>5.2</v>
       </c>
-    </row>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="B80" s="5"/>
+      <c r="N79" s="6"/>
+      <c r="O79" s="5"/>
+    </row>
+    <row r="80" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A80" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B80" s="6">
+        <v>8.5</v>
+      </c>
       <c r="C80" s="5">
-        <f>B80-L80</f>
-        <v>-5.2</v>
+        <f t="shared" si="4"/>
+        <v>3.3</v>
       </c>
       <c r="D80" s="5">
-        <f>B80+L80</f>
-        <v>5.2</v>
-      </c>
-      <c r="E80" s="5"/>
+        <f t="shared" si="5"/>
+        <v>13.7</v>
+      </c>
+      <c r="E80" s="5">
+        <v>3.3</v>
+      </c>
       <c r="F80">
         <v>4</v>
       </c>
-      <c r="G80" s="12"/>
-      <c r="H80" s="12"/>
+      <c r="G80" s="8">
+        <v>3</v>
+      </c>
+      <c r="H80" s="8">
+        <v>5</v>
+      </c>
       <c r="I80" t="s">
         <v>75</v>
       </c>
@@ -9681,23 +9725,36 @@
       <c r="L80" s="5">
         <v>5.2</v>
       </c>
-    </row>
-    <row r="81" spans="2:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="B81" s="5"/>
+      <c r="N80" s="6"/>
+      <c r="O80" s="5"/>
+    </row>
+    <row r="81" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A81" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B81" s="6">
+        <v>8.82</v>
+      </c>
       <c r="C81" s="5">
-        <f>B81-L81</f>
-        <v>-5.2</v>
+        <f t="shared" si="4"/>
+        <v>3.62</v>
       </c>
       <c r="D81" s="5">
-        <f>B81+L81</f>
-        <v>5.2</v>
-      </c>
-      <c r="E81" s="5"/>
+        <f t="shared" si="5"/>
+        <v>14.02</v>
+      </c>
+      <c r="E81" s="5">
+        <v>8.82</v>
+      </c>
       <c r="F81">
         <v>5</v>
       </c>
-      <c r="G81" s="12"/>
-      <c r="H81" s="12"/>
+      <c r="G81" s="8">
+        <v>9</v>
+      </c>
+      <c r="H81" s="8">
+        <v>7</v>
+      </c>
       <c r="I81" t="s">
         <v>75</v>
       </c>
@@ -9710,23 +9767,36 @@
       <c r="L81" s="5">
         <v>5.2</v>
       </c>
-    </row>
-    <row r="82" spans="2:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="B82" s="5"/>
+      <c r="N81" s="6"/>
+      <c r="O81" s="5"/>
+    </row>
+    <row r="82" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A82" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B82" s="6">
+        <v>9.2100000000000009</v>
+      </c>
       <c r="C82" s="5">
-        <f>B82-L82</f>
-        <v>-5.2</v>
+        <f t="shared" si="4"/>
+        <v>4.0100000000000007</v>
       </c>
       <c r="D82" s="5">
-        <f>B82+L82</f>
-        <v>5.2</v>
-      </c>
-      <c r="E82" s="5"/>
+        <f t="shared" si="5"/>
+        <v>14.41</v>
+      </c>
+      <c r="E82" s="5">
+        <v>4.01</v>
+      </c>
       <c r="F82">
         <v>6</v>
       </c>
-      <c r="G82" s="12"/>
-      <c r="H82" s="12"/>
+      <c r="G82" s="8">
+        <v>4</v>
+      </c>
+      <c r="H82" s="8">
+        <v>2</v>
+      </c>
       <c r="I82" t="s">
         <v>75</v>
       </c>
@@ -9739,23 +9809,36 @@
       <c r="L82" s="5">
         <v>5.2</v>
       </c>
-    </row>
-    <row r="83" spans="2:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="B83" s="5"/>
+      <c r="N82" s="6"/>
+      <c r="O82" s="5"/>
+    </row>
+    <row r="83" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A83" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B83" s="6">
+        <v>9.26</v>
+      </c>
       <c r="C83" s="5">
-        <f>B83-L83</f>
-        <v>-5.2</v>
+        <f t="shared" si="4"/>
+        <v>4.0599999999999996</v>
       </c>
       <c r="D83" s="5">
-        <f>B83+L83</f>
-        <v>5.2</v>
-      </c>
-      <c r="E83" s="5"/>
+        <f t="shared" si="5"/>
+        <v>14.46</v>
+      </c>
+      <c r="E83" s="5">
+        <v>9.26</v>
+      </c>
       <c r="F83">
         <v>7</v>
       </c>
-      <c r="G83" s="12"/>
-      <c r="H83" s="12"/>
+      <c r="G83" s="8">
+        <v>10</v>
+      </c>
+      <c r="H83" s="8">
+        <v>3</v>
+      </c>
       <c r="I83" t="s">
         <v>75</v>
       </c>
@@ -9768,23 +9851,36 @@
       <c r="L83" s="5">
         <v>5.2</v>
       </c>
-    </row>
-    <row r="84" spans="2:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="B84" s="5"/>
+      <c r="N83" s="6"/>
+      <c r="O83" s="5"/>
+    </row>
+    <row r="84" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A84" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B84" s="6">
+        <v>9.27</v>
+      </c>
       <c r="C84" s="5">
-        <f>B84-L84</f>
-        <v>-5.2</v>
+        <f t="shared" si="4"/>
+        <v>4.0699999999999994</v>
       </c>
       <c r="D84" s="5">
-        <f>B84+L84</f>
-        <v>5.2</v>
-      </c>
-      <c r="E84" s="5"/>
+        <f t="shared" si="5"/>
+        <v>14.469999999999999</v>
+      </c>
+      <c r="E84" s="5">
+        <v>9.27</v>
+      </c>
       <c r="F84">
         <v>8</v>
       </c>
-      <c r="G84" s="12"/>
-      <c r="H84" s="12"/>
+      <c r="G84" s="8">
+        <v>11</v>
+      </c>
+      <c r="H84" s="8">
+        <v>10</v>
+      </c>
       <c r="I84" t="s">
         <v>75</v>
       </c>
@@ -9797,23 +9893,36 @@
       <c r="L84" s="5">
         <v>5.2</v>
       </c>
-    </row>
-    <row r="85" spans="2:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="B85" s="5"/>
+      <c r="N84" s="6"/>
+      <c r="O84" s="5"/>
+    </row>
+    <row r="85" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A85" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B85" s="6">
+        <v>9.3000000000000007</v>
+      </c>
       <c r="C85" s="5">
-        <f>B85-L85</f>
-        <v>-5.2</v>
+        <f t="shared" si="4"/>
+        <v>4.1000000000000005</v>
       </c>
       <c r="D85" s="5">
-        <f>B85+L85</f>
-        <v>5.2</v>
-      </c>
-      <c r="E85" s="5"/>
+        <f t="shared" si="5"/>
+        <v>14.5</v>
+      </c>
+      <c r="E85" s="5">
+        <v>9.3000000000000007</v>
+      </c>
       <c r="F85">
         <v>9</v>
       </c>
-      <c r="G85" s="12"/>
-      <c r="H85" s="12"/>
+      <c r="G85" s="8">
+        <v>12</v>
+      </c>
+      <c r="H85" s="8">
+        <v>16</v>
+      </c>
       <c r="I85" t="s">
         <v>75</v>
       </c>
@@ -9826,23 +9935,36 @@
       <c r="L85" s="5">
         <v>5.2</v>
       </c>
-    </row>
-    <row r="86" spans="2:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="B86" s="5"/>
+      <c r="N85" s="6"/>
+      <c r="O85" s="5"/>
+    </row>
+    <row r="86" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A86" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B86" s="6">
+        <v>9.52</v>
+      </c>
       <c r="C86" s="5">
-        <f>B86-L86</f>
-        <v>-5.2</v>
+        <f t="shared" si="4"/>
+        <v>4.3199999999999994</v>
       </c>
       <c r="D86" s="5">
-        <f>B86+L86</f>
-        <v>5.2</v>
-      </c>
-      <c r="E86" s="5"/>
+        <f t="shared" si="5"/>
+        <v>14.719999999999999</v>
+      </c>
+      <c r="E86" s="5">
+        <v>4.32</v>
+      </c>
       <c r="F86">
         <v>10</v>
       </c>
-      <c r="G86" s="12"/>
-      <c r="H86" s="12"/>
+      <c r="G86" s="8">
+        <v>5</v>
+      </c>
+      <c r="H86" s="8">
+        <v>17</v>
+      </c>
       <c r="I86" t="s">
         <v>75</v>
       </c>
@@ -9855,23 +9977,36 @@
       <c r="L86" s="5">
         <v>5.2</v>
       </c>
-    </row>
-    <row r="87" spans="2:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="B87" s="5"/>
+      <c r="N86" s="6"/>
+      <c r="O86" s="5"/>
+    </row>
+    <row r="87" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A87" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B87" s="6">
+        <v>10.9</v>
+      </c>
       <c r="C87" s="5">
-        <f>B87-L87</f>
-        <v>-5.2</v>
+        <f t="shared" si="4"/>
+        <v>5.7</v>
       </c>
       <c r="D87" s="5">
-        <f>B87+L87</f>
-        <v>5.2</v>
-      </c>
-      <c r="E87" s="5"/>
+        <f t="shared" si="5"/>
+        <v>16.100000000000001</v>
+      </c>
+      <c r="E87" s="5">
+        <v>10.9</v>
+      </c>
       <c r="F87">
         <v>11</v>
       </c>
-      <c r="G87" s="12"/>
-      <c r="H87" s="12"/>
+      <c r="G87" s="8">
+        <v>13</v>
+      </c>
+      <c r="H87" s="8">
+        <v>11</v>
+      </c>
       <c r="I87" t="s">
         <v>75</v>
       </c>
@@ -9884,23 +10019,36 @@
       <c r="L87" s="5">
         <v>5.2</v>
       </c>
-    </row>
-    <row r="88" spans="2:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="B88" s="5"/>
+      <c r="N87" s="6"/>
+      <c r="O87" s="5"/>
+    </row>
+    <row r="88" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A88" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B88" s="6">
+        <v>11.44</v>
+      </c>
       <c r="C88" s="5">
-        <f>B88-L88</f>
-        <v>-5.2</v>
+        <f t="shared" si="4"/>
+        <v>6.2399999999999993</v>
       </c>
       <c r="D88" s="5">
-        <f>B88+L88</f>
-        <v>5.2</v>
-      </c>
-      <c r="E88" s="5"/>
+        <f t="shared" si="5"/>
+        <v>16.64</v>
+      </c>
+      <c r="E88" s="5">
+        <v>11.44</v>
+      </c>
       <c r="F88">
         <v>12</v>
       </c>
-      <c r="G88" s="12"/>
-      <c r="H88" s="12"/>
+      <c r="G88" s="8">
+        <v>14</v>
+      </c>
+      <c r="H88" s="8">
+        <v>9</v>
+      </c>
       <c r="I88" t="s">
         <v>75</v>
       </c>
@@ -9913,23 +10061,36 @@
       <c r="L88" s="5">
         <v>5.2</v>
       </c>
-    </row>
-    <row r="89" spans="2:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="B89" s="5"/>
+      <c r="N88" s="6"/>
+      <c r="O88" s="5"/>
+    </row>
+    <row r="89" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A89" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B89" s="6">
+        <v>11.89</v>
+      </c>
       <c r="C89" s="5">
-        <f>B89-L89</f>
-        <v>-5.2</v>
+        <f t="shared" si="4"/>
+        <v>6.69</v>
       </c>
       <c r="D89" s="5">
-        <f>B89+L89</f>
-        <v>5.2</v>
-      </c>
-      <c r="E89" s="5"/>
+        <f t="shared" si="5"/>
+        <v>17.09</v>
+      </c>
+      <c r="E89" s="5">
+        <v>6.69</v>
+      </c>
       <c r="F89">
         <v>13</v>
       </c>
-      <c r="G89" s="12"/>
-      <c r="H89" s="12"/>
+      <c r="G89" s="8">
+        <v>6</v>
+      </c>
+      <c r="H89" s="8">
+        <v>15</v>
+      </c>
       <c r="I89" t="s">
         <v>75</v>
       </c>
@@ -9942,23 +10103,36 @@
       <c r="L89" s="5">
         <v>5.2</v>
       </c>
-    </row>
-    <row r="90" spans="2:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="B90" s="5"/>
+      <c r="N89" s="6"/>
+      <c r="O89" s="5"/>
+    </row>
+    <row r="90" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A90" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B90" s="6">
+        <v>12.26</v>
+      </c>
       <c r="C90" s="5">
-        <f>B90-L90</f>
-        <v>-5.2</v>
+        <f t="shared" si="4"/>
+        <v>7.06</v>
       </c>
       <c r="D90" s="5">
-        <f>B90+L90</f>
-        <v>5.2</v>
-      </c>
-      <c r="E90" s="5"/>
+        <f t="shared" si="5"/>
+        <v>17.46</v>
+      </c>
+      <c r="E90" s="5">
+        <v>12.26</v>
+      </c>
       <c r="F90">
         <v>14</v>
       </c>
-      <c r="G90" s="12"/>
-      <c r="H90" s="12"/>
+      <c r="G90" s="8">
+        <v>16</v>
+      </c>
+      <c r="H90" s="8">
+        <v>8</v>
+      </c>
       <c r="I90" t="s">
         <v>75</v>
       </c>
@@ -9971,23 +10145,36 @@
       <c r="L90" s="5">
         <v>5.2</v>
       </c>
-    </row>
-    <row r="91" spans="2:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="B91" s="5"/>
+      <c r="N90" s="6"/>
+      <c r="O90" s="5"/>
+    </row>
+    <row r="91" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A91" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B91" s="6">
+        <v>12.39</v>
+      </c>
       <c r="C91" s="5">
-        <f>B91-L91</f>
-        <v>-5.2</v>
+        <f t="shared" si="4"/>
+        <v>7.19</v>
       </c>
       <c r="D91" s="5">
-        <f>B91+L91</f>
-        <v>5.2</v>
-      </c>
-      <c r="E91" s="5"/>
+        <f t="shared" si="5"/>
+        <v>17.59</v>
+      </c>
+      <c r="E91" s="5">
+        <v>7.19</v>
+      </c>
       <c r="F91">
         <v>15</v>
       </c>
-      <c r="G91" s="12"/>
-      <c r="H91" s="12"/>
+      <c r="G91" s="8">
+        <v>7</v>
+      </c>
+      <c r="H91" s="8">
+        <v>12</v>
+      </c>
       <c r="I91" t="s">
         <v>75</v>
       </c>
@@ -10000,23 +10187,36 @@
       <c r="L91" s="5">
         <v>5.2</v>
       </c>
-    </row>
-    <row r="92" spans="2:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="B92" s="5"/>
+      <c r="N91" s="6"/>
+      <c r="O91" s="5"/>
+    </row>
+    <row r="92" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A92" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B92" s="6">
+        <v>12.74</v>
+      </c>
       <c r="C92" s="5">
-        <f>B92-L92</f>
-        <v>-5.2</v>
+        <f t="shared" si="4"/>
+        <v>7.54</v>
       </c>
       <c r="D92" s="5">
-        <f>B92+L92</f>
-        <v>5.2</v>
-      </c>
-      <c r="E92" s="5"/>
+        <f t="shared" si="5"/>
+        <v>17.940000000000001</v>
+      </c>
+      <c r="E92" s="5">
+        <v>12.74</v>
+      </c>
       <c r="F92">
         <v>16</v>
       </c>
-      <c r="G92" s="12"/>
-      <c r="H92" s="12"/>
+      <c r="G92" s="8">
+        <v>17</v>
+      </c>
+      <c r="H92" s="8">
+        <v>13</v>
+      </c>
       <c r="I92" t="s">
         <v>75</v>
       </c>
@@ -10029,23 +10229,36 @@
       <c r="L92" s="5">
         <v>5.2</v>
       </c>
-    </row>
-    <row r="93" spans="2:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="B93" s="5"/>
+      <c r="N92" s="6"/>
+      <c r="O92" s="5"/>
+    </row>
+    <row r="93" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A93" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B93" s="6">
+        <v>12.78</v>
+      </c>
       <c r="C93" s="5">
-        <f>B93-L93</f>
-        <v>-5.2</v>
+        <f t="shared" si="4"/>
+        <v>7.5799999999999992</v>
       </c>
       <c r="D93" s="5">
-        <f>B93+L93</f>
-        <v>5.2</v>
-      </c>
-      <c r="E93" s="5"/>
+        <f t="shared" si="5"/>
+        <v>17.98</v>
+      </c>
+      <c r="E93" s="5">
+        <v>17.98</v>
+      </c>
       <c r="F93">
         <v>17</v>
       </c>
-      <c r="G93" s="12"/>
-      <c r="H93" s="12"/>
+      <c r="G93" s="8">
+        <v>22</v>
+      </c>
+      <c r="H93" s="8">
+        <v>20</v>
+      </c>
       <c r="I93" t="s">
         <v>75</v>
       </c>
@@ -10058,23 +10271,36 @@
       <c r="L93" s="5">
         <v>5.2</v>
       </c>
-    </row>
-    <row r="94" spans="2:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="B94" s="5"/>
+      <c r="N93" s="6"/>
+      <c r="O93" s="5"/>
+    </row>
+    <row r="94" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A94" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B94" s="6">
+        <v>13.64</v>
+      </c>
       <c r="C94" s="5">
-        <f>B94-L94</f>
-        <v>-5.2</v>
+        <f t="shared" si="4"/>
+        <v>8.4400000000000013</v>
       </c>
       <c r="D94" s="5">
-        <f>B94+L94</f>
-        <v>5.2</v>
-      </c>
-      <c r="E94" s="5"/>
+        <f t="shared" si="5"/>
+        <v>18.84</v>
+      </c>
+      <c r="E94" s="5">
+        <v>13.64</v>
+      </c>
       <c r="F94">
         <v>18</v>
       </c>
-      <c r="G94" s="12"/>
-      <c r="H94" s="12"/>
+      <c r="G94" s="8">
+        <v>18</v>
+      </c>
+      <c r="H94" s="8">
+        <v>14</v>
+      </c>
       <c r="I94" t="s">
         <v>75</v>
       </c>
@@ -10087,23 +10313,36 @@
       <c r="L94" s="5">
         <v>5.2</v>
       </c>
-    </row>
-    <row r="95" spans="2:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="B95" s="5"/>
+      <c r="N94" s="6"/>
+      <c r="O94" s="5"/>
+    </row>
+    <row r="95" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A95" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B95" s="6">
+        <v>13.75</v>
+      </c>
       <c r="C95" s="5">
-        <f>B95-L95</f>
-        <v>-5.2</v>
+        <f t="shared" si="4"/>
+        <v>8.5500000000000007</v>
       </c>
       <c r="D95" s="5">
-        <f>B95+L95</f>
-        <v>5.2</v>
-      </c>
-      <c r="E95" s="5"/>
+        <f t="shared" si="5"/>
+        <v>18.95</v>
+      </c>
+      <c r="E95" s="5">
+        <v>18.95</v>
+      </c>
       <c r="F95">
         <v>19</v>
       </c>
-      <c r="G95" s="12"/>
-      <c r="H95" s="12"/>
+      <c r="G95" s="8">
+        <v>23</v>
+      </c>
+      <c r="H95" s="8">
+        <v>19</v>
+      </c>
       <c r="I95" t="s">
         <v>75</v>
       </c>
@@ -10116,23 +10355,36 @@
       <c r="L95" s="5">
         <v>5.2</v>
       </c>
-    </row>
-    <row r="96" spans="2:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="B96" s="5"/>
+      <c r="N95" s="6"/>
+      <c r="O95" s="5"/>
+    </row>
+    <row r="96" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A96" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B96" s="6">
+        <v>14.11</v>
+      </c>
       <c r="C96" s="5">
-        <f>B96-L96</f>
-        <v>-5.2</v>
+        <f t="shared" si="4"/>
+        <v>8.91</v>
       </c>
       <c r="D96" s="5">
-        <f>B96+L96</f>
-        <v>5.2</v>
-      </c>
-      <c r="E96" s="5"/>
+        <f t="shared" si="5"/>
+        <v>19.309999999999999</v>
+      </c>
+      <c r="E96" s="5">
+        <v>19.309999999999999</v>
+      </c>
       <c r="F96">
         <v>20</v>
       </c>
-      <c r="G96" s="12"/>
-      <c r="H96" s="12"/>
+      <c r="G96" s="8">
+        <v>24</v>
+      </c>
+      <c r="H96" s="8">
+        <v>18</v>
+      </c>
       <c r="I96" t="s">
         <v>75</v>
       </c>
@@ -10145,23 +10397,36 @@
       <c r="L96" s="5">
         <v>5.2</v>
       </c>
-    </row>
-    <row r="97" spans="2:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="B97" s="5"/>
+      <c r="N96" s="6"/>
+      <c r="O96" s="5"/>
+    </row>
+    <row r="97" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A97" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B97" s="6">
+        <v>15.58</v>
+      </c>
       <c r="C97" s="5">
-        <f>B97-L97</f>
-        <v>-5.2</v>
+        <f t="shared" si="4"/>
+        <v>10.379999999999999</v>
       </c>
       <c r="D97" s="5">
-        <f>B97+L97</f>
-        <v>5.2</v>
-      </c>
-      <c r="E97" s="5"/>
+        <f t="shared" si="5"/>
+        <v>20.78</v>
+      </c>
+      <c r="E97" s="5">
+        <v>15.58</v>
+      </c>
       <c r="F97">
         <v>21</v>
       </c>
-      <c r="G97" s="12"/>
-      <c r="H97" s="12"/>
+      <c r="G97" s="8">
+        <v>19</v>
+      </c>
+      <c r="H97" s="8">
+        <v>25</v>
+      </c>
       <c r="I97" t="s">
         <v>75</v>
       </c>
@@ -10174,23 +10439,36 @@
       <c r="L97" s="5">
         <v>5.2</v>
       </c>
-    </row>
-    <row r="98" spans="2:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="B98" s="5"/>
+      <c r="N97" s="6"/>
+      <c r="O97" s="5"/>
+    </row>
+    <row r="98" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A98" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B98" s="6">
+        <v>16.14</v>
+      </c>
       <c r="C98" s="5">
-        <f>B98-L98</f>
-        <v>-5.2</v>
+        <f t="shared" ref="C98:C101" si="6">B98-L98</f>
+        <v>10.940000000000001</v>
       </c>
       <c r="D98" s="5">
-        <f>B98+L98</f>
-        <v>5.2</v>
-      </c>
-      <c r="E98" s="5"/>
+        <f t="shared" si="5"/>
+        <v>21.34</v>
+      </c>
+      <c r="E98" s="5">
+        <v>16.14</v>
+      </c>
       <c r="F98">
         <v>22</v>
       </c>
-      <c r="G98" s="12"/>
-      <c r="H98" s="12"/>
+      <c r="G98" s="8">
+        <v>20</v>
+      </c>
+      <c r="H98" s="8">
+        <v>24</v>
+      </c>
       <c r="I98" t="s">
         <v>75</v>
       </c>
@@ -10203,23 +10481,36 @@
       <c r="L98" s="5">
         <v>5.2</v>
       </c>
-    </row>
-    <row r="99" spans="2:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="B99" s="5"/>
+      <c r="N98" s="6"/>
+      <c r="O98" s="5"/>
+    </row>
+    <row r="99" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A99" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B99" s="6">
+        <v>16.88</v>
+      </c>
       <c r="C99" s="5">
-        <f>B99-L99</f>
-        <v>-5.2</v>
+        <f t="shared" si="6"/>
+        <v>11.68</v>
       </c>
       <c r="D99" s="5">
-        <f>B99+L99</f>
-        <v>5.2</v>
-      </c>
-      <c r="E99" s="5"/>
+        <f t="shared" si="5"/>
+        <v>22.08</v>
+      </c>
+      <c r="E99" s="5">
+        <v>16.88</v>
+      </c>
       <c r="F99">
         <v>23</v>
       </c>
-      <c r="G99" s="12"/>
-      <c r="H99" s="12"/>
+      <c r="G99" s="8">
+        <v>21</v>
+      </c>
+      <c r="H99" s="8">
+        <v>23</v>
+      </c>
       <c r="I99" t="s">
         <v>75</v>
       </c>
@@ -10232,23 +10523,36 @@
       <c r="L99" s="5">
         <v>5.2</v>
       </c>
-    </row>
-    <row r="100" spans="2:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="B100" s="5"/>
+      <c r="N99" s="6"/>
+      <c r="O99" s="5"/>
+    </row>
+    <row r="100" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A100" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B100" s="6">
+        <v>17.329999999999998</v>
+      </c>
       <c r="C100" s="5">
-        <f>B100-L100</f>
-        <v>-5.2</v>
+        <f t="shared" si="6"/>
+        <v>12.129999999999999</v>
       </c>
       <c r="D100" s="5">
-        <f>B100+L100</f>
-        <v>5.2</v>
-      </c>
-      <c r="E100" s="5"/>
+        <f t="shared" si="5"/>
+        <v>22.529999999999998</v>
+      </c>
+      <c r="E100" s="5">
+        <v>12.13</v>
+      </c>
       <c r="F100">
         <v>24</v>
       </c>
-      <c r="G100" s="12"/>
-      <c r="H100" s="12"/>
+      <c r="G100" s="8">
+        <v>15</v>
+      </c>
+      <c r="H100" s="8">
+        <v>21</v>
+      </c>
       <c r="I100" t="s">
         <v>75</v>
       </c>
@@ -10261,23 +10565,36 @@
       <c r="L100" s="5">
         <v>5.2</v>
       </c>
-    </row>
-    <row r="101" spans="2:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="B101" s="5"/>
+      <c r="N100" s="6"/>
+      <c r="O100" s="5"/>
+    </row>
+    <row r="101" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A101" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B101" s="6">
+        <v>17.54</v>
+      </c>
       <c r="C101" s="5">
-        <f>B101-L101</f>
-        <v>-5.2</v>
+        <f t="shared" si="6"/>
+        <v>12.34</v>
       </c>
       <c r="D101" s="5">
-        <f>B101+L101</f>
-        <v>5.2</v>
-      </c>
-      <c r="E101" s="5"/>
+        <f t="shared" si="5"/>
+        <v>22.74</v>
+      </c>
+      <c r="E101" s="5">
+        <v>22.74</v>
+      </c>
       <c r="F101">
         <v>25</v>
       </c>
-      <c r="G101" s="12"/>
-      <c r="H101" s="12"/>
+      <c r="G101" s="8">
+        <v>25</v>
+      </c>
+      <c r="H101" s="8">
+        <v>22</v>
+      </c>
       <c r="I101" t="s">
         <v>75</v>
       </c>
@@ -10290,10 +10607,16 @@
       <c r="L101" s="5">
         <v>5.2</v>
       </c>
+      <c r="N101" s="6"/>
+      <c r="O101" s="5"/>
+    </row>
+    <row r="102" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="N102" s="6"/>
+      <c r="O102" s="5"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="N27:O51">
-    <sortCondition ref="O27:O51"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="N78:O102">
+    <sortCondition ref="O102"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="88" orientation="landscape" r:id="rId1"/>

</xml_diff>